<commit_message>
T2 v2: review round 1, five department lines for the per-employee table, 13 rows and 79 points
The first review read the 27-row file and raised two findings, both accepted.
A row per current employee was 156 requirements over the 25-criterion limit,
and the measurement-date sentence was an ask no row read. Both are out of the
memo and barred with a control each. The memo asks for the two totals and the
PTO hours and PTO liability of five lines, Sales and Marketing joined because
Marketing alone is a figure the load already carries right.

The engine reads a line by a whole-cell name or a prose line that opens on it,
never off an employee row. Battery 520 of 520 on 40 snapshots, 70 of 70
controls red, the golden 79 of 79, P0 and P1 at 1 point. The record writers
now read the battery and the re-scoring off the scripts on every write.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ECfiP9fiqeMK3tptE1VHjz
</commit_message>
<xml_diff>
--- a/tasks/HR_Troutly_T2v2_pto_liability_close/03_show_your_work.xlsx
+++ b/tasks/HR_Troutly_T2v2_pto_liability_close/03_show_your_work.xlsx
@@ -707,7 +707,7 @@
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>57 active rows, the loaded policies, six of them wrong, and the loaded balances the run brings to the schedule.</t>
+          <t>57 active rows, the loaded policies, six of them wrong, and the loaded balances. Read, never written.</t>
         </is>
       </c>
     </row>
@@ -722,7 +722,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D33"/>
+  <dimension ref="A1:D19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -813,11 +813,11 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>States, on the PTO liability page, a balance of 64.62 hours for Mikelle Hosana, TRT-0005.</t>
+          <t>States, on the PTO liability page, PTO hours of 297.79 for Customer Success.</t>
         </is>
       </c>
       <c r="C5" s="2" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
@@ -831,11 +831,11 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>States, on the PTO liability page, a balance of 64.62 hours for Krystale Jumawan, TRT-0009.</t>
+          <t>States, on the PTO liability page, a PTO liability of $12,627.20 for Customer Success.</t>
         </is>
       </c>
       <c r="C6" s="2" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
@@ -849,7 +849,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>States, on the PTO liability page, a balance of 18.46 hours for Jessica Ko, TRT-0012.</t>
+          <t>States, on the PTO liability page, PTO hours of 558.31 for Engineering.</t>
         </is>
       </c>
       <c r="C7" s="2" t="n">
@@ -867,7 +867,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>States, on the PTO liability page, a balance of 60.00 hours for Marisela Thornbury, TRT-0018.</t>
+          <t>States, on the PTO liability page, a PTO liability of $41,542.16 for Engineering.</t>
         </is>
       </c>
       <c r="C8" s="2" t="n">
@@ -885,11 +885,11 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>States, on the PTO liability page, a balance of 42.46 hours for Edith Bustamante, TRT-0021.</t>
+          <t>States, on the PTO liability page, PTO hours of 121.53 for Finance and Corporate.</t>
         </is>
       </c>
       <c r="C9" s="2" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
@@ -903,11 +903,11 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>States, on the PTO liability page, a balance of 58.46 hours for Rohan Iyer, TRT-0014.</t>
+          <t>States, on the PTO liability page, a PTO liability of $8,187.68 for Finance and Corporate.</t>
         </is>
       </c>
       <c r="C10" s="2" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
@@ -921,11 +921,11 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>States, on the PTO liability page, a balance of 58.46 hours for Maeve Oyinlola, TRT-0023.</t>
+          <t>States, on the PTO liability page, PTO hours of 170.50 for Product.</t>
         </is>
       </c>
       <c r="C11" s="2" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
@@ -939,11 +939,11 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>States, on the PTO liability page, a balance of 26.46 hours for Zephyr Adebayo, TRT-0031.</t>
+          <t>States, on the PTO liability page, a PTO liability of $10,984.34 for Product.</t>
         </is>
       </c>
       <c r="C12" s="2" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
@@ -957,11 +957,11 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>States, on the PTO liability page, a balance of 50.46 hours for Emeka Thorsen, TRT-0029.</t>
+          <t>States, on the PTO liability page, PTO hours of 374.04 for Sales and Marketing.</t>
         </is>
       </c>
       <c r="C13" s="2" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
@@ -975,11 +975,11 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>States, on the PTO liability page, a balance of 58.46 hours for Ilse Van der Kolk, TRT-0040.</t>
+          <t>States, on the PTO liability page, a PTO liability of $19,398.16 for Sales and Marketing.</t>
         </is>
       </c>
       <c r="C14" s="2" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
@@ -988,318 +988,66 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="2" t="n">
-        <v>14</v>
-      </c>
-      <c r="B15" s="2" t="inlineStr">
-        <is>
-          <t>States, on the PTO liability page, a balance of 51.87 hours for Samuel Burkenham, TRT-0071.</t>
-        </is>
-      </c>
-      <c r="C15" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="D15" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
+      <c r="A15" s="2" t="n"/>
+      <c r="B15" s="2" t="n"/>
+      <c r="C15" s="2" t="n"/>
+      <c r="D15" s="2" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="2" t="n">
-        <v>15</v>
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>States, on the PTO liability page, a balance of 6.71 hours for Priyamvada Raghunath, TRT-0051.</t>
-        </is>
-      </c>
-      <c r="C16" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="D16" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
+          <t>Row 2 reads the total of all 52 liabilities, the one number every rule feeds, and it matches the schedule's only if every entry is right. Row 3 reads the same population on the hours axis.</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="n"/>
+      <c r="D16" s="2" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="2" t="n">
-        <v>16</v>
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>States, on the PTO liability page, a balance of 24.96 hours for Wren Takahashi-Bell, TRT-0079.</t>
-        </is>
-      </c>
-      <c r="C17" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="D17" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
+          <t>Rows 4 to 13 read the five lines the request asks for, each line's hours and dollars. Every line figure is one the load carries wrong, so a response that copies the report earns none of them and a response that applies the rules earns them all.</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="n"/>
+      <c r="D17" s="2" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="2" t="n">
-        <v>17</v>
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>States, on the PTO liability page, a balance of 40.96 hours for Callum Oyelaran, TRT-0058.</t>
-        </is>
-      </c>
-      <c r="C18" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="D18" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
+          <t>Each line figure carries the dollars it moves off the load, banded 7 where the figure moves $2,000.00 or more, 6 where the figure moves $800.00 or more, 5 where the figure moves $250.00 or more, 4 where the figure moves $80.00 or more and 3 below that. Sales and Marketing are one line because Marketing alone is a figure the load already carries right.</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="n"/>
+      <c r="D18" s="2" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="2" t="n">
-        <v>18</v>
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>States, on the PTO liability page, a balance of 18.71 hours for Desmond Achterberg, TRT-0083.</t>
-        </is>
-      </c>
-      <c r="C19" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="D19" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="2" t="n">
-        <v>19</v>
-      </c>
-      <c r="B20" s="2" t="inlineStr">
-        <is>
-          <t>States, on the PTO liability page, a balance of 6.15 hours for Simone Okonkwo, TRT-0153.</t>
-        </is>
-      </c>
-      <c r="C20" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="D20" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="2" t="n">
-        <v>20</v>
-      </c>
-      <c r="B21" s="2" t="inlineStr">
-        <is>
-          <t>States, on the PTO liability page, an hourly rate of $44.2308 for Simone Okonkwo, TRT-0153.</t>
-        </is>
-      </c>
-      <c r="C21" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="D21" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="2" t="n">
-        <v>21</v>
-      </c>
-      <c r="B22" s="2" t="inlineStr">
-        <is>
-          <t>States, on the PTO liability page, a balance of 34.46 hours for Oren Kastellanos, TRT-0043.</t>
-        </is>
-      </c>
-      <c r="C22" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="D22" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="2" t="n">
-        <v>22</v>
-      </c>
-      <c r="B23" s="2" t="inlineStr">
-        <is>
-          <t>States, on the PTO liability page, an hourly rate of $56.7308 for Yolanda Featherstone, TRT-0088.</t>
-        </is>
-      </c>
-      <c r="C23" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="D23" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="2" t="n">
-        <v>23</v>
-      </c>
-      <c r="B24" s="2" t="inlineStr">
-        <is>
-          <t>States, on the PTO liability page, a balance of 3.08 hours for Rafael Ibarra, TRT-0155.</t>
-        </is>
-      </c>
-      <c r="C24" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="D24" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="2" t="n">
-        <v>24</v>
-      </c>
-      <c r="B25" s="2" t="inlineStr">
-        <is>
-          <t>States, on the PTO liability page, an hourly rate of $27.0673 for Rafael Ibarra, TRT-0155.</t>
-        </is>
-      </c>
-      <c r="C25" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="D25" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="2" t="n">
-        <v>25</v>
-      </c>
-      <c r="B26" s="2" t="inlineStr">
-        <is>
-          <t>States, on the PTO liability page, a balance of 29.60 hours for Beatriz Quintanilla, TRT-0141.</t>
-        </is>
-      </c>
-      <c r="C26" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="D26" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="2" t="n">
-        <v>26</v>
-      </c>
-      <c r="B27" s="2" t="inlineStr">
-        <is>
-          <t>States, on the PTO liability page, an hourly rate of $71.2500 for Belaviv Luk, TRT-0117.</t>
-        </is>
-      </c>
-      <c r="C27" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="D27" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="2" t="n">
-        <v>27</v>
-      </c>
-      <c r="B28" s="2" t="inlineStr">
-        <is>
-          <t>States, on the PTO liability page, an hourly rate of $29.3269 for Delphine Marchetti, TRT-0096.</t>
-        </is>
-      </c>
-      <c r="C28" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="D28" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="2" t="n"/>
-      <c r="B29" s="2" t="n"/>
-      <c r="C29" s="2" t="n"/>
-      <c r="D29" s="2" t="n"/>
-    </row>
-    <row r="30">
-      <c r="A30" s="2" t="inlineStr">
-        <is>
-          <t>Note</t>
-        </is>
-      </c>
-      <c r="B30" s="2" t="inlineStr">
-        <is>
-          <t>Row 2 grades every rule across the whole group at once. It reads the total of all 52 liabilities, the one number every cell feeds, and it matches the schedule's only if every entry is right. Row 3 reads the same population on the hours axis.</t>
-        </is>
-      </c>
-      <c r="C30" s="2" t="n"/>
-      <c r="D30" s="2" t="n"/>
-    </row>
-    <row r="31">
-      <c r="A31" s="2" t="inlineStr">
-        <is>
-          <t>Note</t>
-        </is>
-      </c>
-      <c r="B31" s="2" t="inlineStr">
-        <is>
-          <t>Rows 4 to 27 each read one cell the load carries wrong, 19 balances and 5 rates over 22 employees. A cell is graded only where the figure the world gives is not the figure the load carries, so a response that copies the report earns none of them and a response that applies the rules earns them all.</t>
-        </is>
-      </c>
-      <c r="C31" s="2" t="n"/>
-      <c r="D31" s="2" t="n"/>
-    </row>
-    <row r="32">
-      <c r="A32" s="2" t="inlineStr">
-        <is>
-          <t>Note</t>
-        </is>
-      </c>
-      <c r="B32" s="2" t="inlineStr">
-        <is>
-          <t>Each of those rows carries the dollars it moves, $23,539.62 in all, banded 7 where the cell moves $2,000.00 or more, 6 where the cell moves $800.00 or more, 5 where the cell moves $250.00 or more, 4 where the cell moves $80.00 or more and 3 below that. Nothing in the set grades the absence of content, so a response that prints all 52 employees rather than the 22 the load has wrong loses nothing by it.</t>
-        </is>
-      </c>
-      <c r="C32" s="2" t="n"/>
-      <c r="D32" s="2" t="n"/>
-    </row>
-    <row r="33">
-      <c r="A33" s="2" t="inlineStr">
-        <is>
-          <t>Note</t>
-        </is>
-      </c>
-      <c r="B33" s="2" t="inlineStr">
-        <is>
-          <t>Row 1 is the only row that is not a determination. It carries 1 point of 143, which is the whole of what a response earns for publishing a page with the wrong numbers on it.</t>
-        </is>
-      </c>
-      <c r="C33" s="2" t="n"/>
-      <c r="D33" s="2" t="n"/>
+          <t>Row 1 is the only row that is not a determination. It carries 1 point of 79, which is the whole of what a response earns for publishing a page with the wrong numbers on it.</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="n"/>
+      <c r="D19" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1430,24 +1178,24 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>The page</t>
+          <t>The lines</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>PTO Liability - 08/31/2026. The summary above the table, seven columns, 52 rows keyed by ID, published.</t>
+          <t>The 52 employees summed by department onto the request's five lines, Sales and Marketing together. Customer Success 297.79 hours and $12,627.20. Engineering 558.31 hours and $41,542.16. Finance and Corporate 121.53 hours and $8,187.68. Product 170.50 hours and $10,984.34. Sales and Marketing 374.04 hours and $19,398.16.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>BambooHR</t>
+          <t>The page</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Six policies reassigned and 44 left as loaded. 17 balances moved and 33 left as loaded. Rows created for TRT-0153 and TRT-0155 with the 80-hour policy.</t>
+          <t>PTO Liability - 08/31/2026. The two totals, then one table of the five lines, published.</t>
         </is>
       </c>
     </row>

</xml_diff>